<commit_message>
Doc/content sync: weekly FB digest runs, Beelining project note, landing page redesign notes
Weekly FB digest updates through Sep 6 run (Sep 7-20 scheduled), Caren
Cooper meeting confirmed for Oct 1 in KEY_PEOPLE_CONTACTS.md, standalone
Beelining PWA project note in CLAUDE.md, and handoff notes from a
landing-page redesign design-review session.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Legacy_Submitter_Outreach_Tracker.xlsx
+++ b/Legacy_Submitter_Outreach_Tracker.xlsx
@@ -14,8 +14,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -68,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -81,6 +82,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -520,12 +524,18 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="n">
+        <v>46244</v>
+      </c>
       <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTED 2026-09-03: tracker wrongly showed Not yet contacted — actually emailed Mon Aug 10, 2026 3:00 PM (generic legacy template, old hello@savethehives.org signature). Discovered when a duplicate send was scheduled for today; that duplicate was cancelled. IMPORTANT CONTEXT: Falco has a real prior relationship with Ronnie from Mar 2015 — he is/was president of the Haarlem Beekeepers Association (Netherlands, blog ImkerijHaarlem.nl) and wanted to onboard his whole association onto the registration system. Ronnie replied enthusiastically at the time. A personalized follow-up (not the generic template) referencing this history is being drafted separately — do not send the generic template to Falco again.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1726,14 +1736,16 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="n">
+        <v>46248</v>
+      </c>
       <c r="P18" s="2" t="n"/>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>Draft created in Gmail 2026-08-11 (trimmed template, no [PERSONAL NOTE], all hive links included), not yet sent.</t>
+          <t>CORRECTED 2026-09-03: tracker wrongly showed Not yet contacted — actually emailed Fri Aug 14, 2026 ~9:39 AM (generic legacy template), no reply yet. Discovered during pre-send duplicate check; pulled from today's batch to avoid re-sending the same email. No known special history — fine to fold into a later, differently-worded follow-up round rather than urgent personalized outreach.</t>
         </is>
       </c>
     </row>
@@ -2225,14 +2237,16 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O25" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O25" s="6" t="n">
+        <v>46248</v>
+      </c>
       <c r="P25" s="2" t="n"/>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>Draft created in Gmail 2026-08-11 (trimmed template, no [PERSONAL NOTE], all hive links included), not yet sent.</t>
+          <t>CORRECTED 2026-09-03: tracker wrongly showed Not yet contacted — actually emailed Fri Aug 14, 2026 1:00 PM (generic legacy template), no reply yet. Discovered during pre-send duplicate check; pulled from today's batch to avoid re-sending the same email. No known special history — fine to fold into a later, differently-worded follow-up round rather than urgent personalized outreach.</t>
         </is>
       </c>
     </row>
@@ -2367,10 +2381,12 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O27" s="2" t="n"/>
+          <t>Emailed - Bounced</t>
+        </is>
+      </c>
+      <c r="O27" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P27" s="2" t="n"/>
       <c r="Q27" s="2" t="n"/>
     </row>
@@ -2440,10 +2456,12 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O28" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O28" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P28" s="2" t="n"/>
       <c r="Q28" s="2" t="inlineStr">
         <is>
@@ -2517,10 +2535,12 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O29" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O29" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P29" s="2" t="n"/>
       <c r="Q29" s="2" t="n"/>
     </row>
@@ -2586,10 +2606,12 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O30" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P30" s="2" t="n"/>
       <c r="Q30" s="2" t="n"/>
     </row>
@@ -2647,10 +2669,12 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O31" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O31" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P31" s="2" t="n"/>
       <c r="Q31" s="2" t="n"/>
     </row>
@@ -2720,10 +2744,12 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O32" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O32" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P32" s="2" t="n"/>
       <c r="Q32" s="2" t="inlineStr">
         <is>
@@ -2797,10 +2823,12 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O33" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P33" s="2" t="n"/>
       <c r="Q33" s="2" t="n"/>
     </row>
@@ -2858,10 +2886,12 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O34" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O34" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P34" s="2" t="n"/>
       <c r="Q34" s="2" t="n"/>
     </row>
@@ -2931,10 +2961,12 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O35" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O35" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P35" s="2" t="n"/>
       <c r="Q35" s="2" t="n"/>
     </row>
@@ -2992,10 +3024,12 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O36" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O36" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P36" s="2" t="n"/>
       <c r="Q36" s="2" t="n"/>
     </row>
@@ -3053,10 +3087,12 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O37" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O37" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P37" s="2" t="n"/>
       <c r="Q37" s="2" t="n"/>
     </row>
@@ -3126,10 +3162,12 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="n"/>
+          <t>Emailed - Bounced</t>
+        </is>
+      </c>
+      <c r="O38" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P38" s="2" t="n"/>
       <c r="Q38" s="2" t="inlineStr">
         <is>
@@ -3203,10 +3241,12 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O39" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O39" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P39" s="2" t="n"/>
       <c r="Q39" s="2" t="n"/>
     </row>
@@ -3276,10 +3316,12 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O40" s="2" t="n"/>
+          <t>Emailed - Bounced</t>
+        </is>
+      </c>
+      <c r="O40" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P40" s="2" t="n"/>
       <c r="Q40" s="2" t="inlineStr">
         <is>
@@ -3353,10 +3395,12 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O41" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O41" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P41" s="2" t="n"/>
       <c r="Q41" s="2" t="n"/>
     </row>
@@ -3426,10 +3470,12 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O42" s="2" t="n"/>
+          <t>Emailed - Bounced</t>
+        </is>
+      </c>
+      <c r="O42" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P42" s="2" t="n"/>
       <c r="Q42" s="2" t="inlineStr">
         <is>
@@ -3503,10 +3549,12 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O43" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O43" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P43" s="2" t="n"/>
       <c r="Q43" s="2" t="inlineStr">
         <is>
@@ -3580,10 +3628,12 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O44" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O44" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P44" s="2" t="n"/>
       <c r="Q44" s="2" t="n"/>
     </row>
@@ -3653,10 +3703,12 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O45" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O45" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P45" s="2" t="n"/>
       <c r="Q45" s="2" t="n"/>
     </row>
@@ -3726,10 +3778,12 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O46" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O46" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P46" s="2" t="n"/>
       <c r="Q46" s="2" t="n"/>
     </row>
@@ -3787,10 +3841,12 @@
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O47" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O47" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P47" s="2" t="n"/>
       <c r="Q47" s="2" t="n"/>
     </row>
@@ -3860,10 +3916,12 @@
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O48" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O48" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P48" s="2" t="n"/>
       <c r="Q48" s="2" t="inlineStr">
         <is>
@@ -3990,10 +4048,12 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O50" s="2" t="n"/>
+          <t>Emailed - Bounced</t>
+        </is>
+      </c>
+      <c r="O50" s="6" t="n">
+        <v>46268</v>
+      </c>
       <c r="P50" s="2" t="n"/>
       <c r="Q50" s="2" t="inlineStr">
         <is>
@@ -4067,10 +4127,12 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O51" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O51" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P51" s="2" t="n"/>
       <c r="Q51" s="2" t="inlineStr">
         <is>
@@ -4144,10 +4206,12 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O52" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O52" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P52" s="2" t="n"/>
       <c r="Q52" s="2" t="inlineStr">
         <is>
@@ -4221,10 +4285,12 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O53" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O53" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P53" s="2" t="n"/>
       <c r="Q53" s="2" t="n"/>
     </row>
@@ -4282,10 +4348,12 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O54" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O54" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P54" s="2" t="n"/>
       <c r="Q54" s="2" t="n"/>
     </row>
@@ -4355,10 +4423,12 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O55" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O55" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P55" s="2" t="n"/>
       <c r="Q55" s="2" t="n"/>
     </row>
@@ -4428,10 +4498,12 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O56" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O56" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P56" s="2" t="n"/>
       <c r="Q56" s="2" t="n"/>
     </row>
@@ -4501,10 +4573,12 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O57" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O57" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P57" s="2" t="n"/>
       <c r="Q57" s="2" t="n"/>
     </row>
@@ -4574,10 +4648,12 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O58" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O58" s="6" t="n">
+        <v>46272</v>
+      </c>
       <c r="P58" s="2" t="n"/>
       <c r="Q58" s="2" t="inlineStr">
         <is>
@@ -4651,10 +4727,14 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O59" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P59" s="2" t="n"/>
       <c r="Q59" s="2" t="inlineStr">
         <is>
@@ -4716,10 +4796,14 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O60" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P60" s="2" t="n"/>
       <c r="Q60" s="2" t="n"/>
     </row>
@@ -4785,10 +4869,14 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O61" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P61" s="2" t="n"/>
       <c r="Q61" s="2" t="inlineStr">
         <is>
@@ -4862,10 +4950,14 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O62" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P62" s="2" t="n"/>
       <c r="Q62" s="2" t="n"/>
     </row>
@@ -4935,10 +5027,14 @@
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O63" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P63" s="2" t="n"/>
       <c r="Q63" s="2" t="inlineStr">
         <is>
@@ -5012,10 +5108,14 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O64" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P64" s="2" t="n"/>
       <c r="Q64" s="2" t="inlineStr">
         <is>
@@ -5089,10 +5189,14 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O65" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P65" s="2" t="n"/>
       <c r="Q65" s="2" t="n"/>
     </row>
@@ -5162,10 +5266,14 @@
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O66" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P66" s="2" t="n"/>
       <c r="Q66" s="2" t="n"/>
     </row>
@@ -5223,10 +5331,14 @@
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O67" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P67" s="2" t="n"/>
       <c r="Q67" s="2" t="n"/>
     </row>
@@ -5296,10 +5408,14 @@
       </c>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O68" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P68" s="2" t="n"/>
       <c r="Q68" s="2" t="n"/>
     </row>
@@ -5369,10 +5485,14 @@
       </c>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O69" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P69" s="2" t="n"/>
       <c r="Q69" s="2" t="inlineStr">
         <is>
@@ -5446,10 +5566,14 @@
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O70" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P70" s="2" t="n"/>
       <c r="Q70" s="2" t="n"/>
     </row>
@@ -5519,10 +5643,14 @@
       </c>
       <c r="N71" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O71" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P71" s="2" t="n"/>
       <c r="Q71" s="2" t="n"/>
     </row>
@@ -5592,10 +5720,14 @@
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O72" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P72" s="2" t="n"/>
       <c r="Q72" s="2" t="n"/>
     </row>
@@ -5653,10 +5785,14 @@
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O73" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P73" s="2" t="n"/>
       <c r="Q73" s="2" t="inlineStr">
         <is>
@@ -5718,10 +5854,14 @@
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O74" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P74" s="2" t="n"/>
       <c r="Q74" s="2" t="n"/>
     </row>
@@ -5787,10 +5927,14 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O75" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P75" s="2" t="n"/>
       <c r="Q75" s="2" t="inlineStr">
         <is>
@@ -5864,10 +6008,14 @@
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O76" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P76" s="2" t="n"/>
       <c r="Q76" s="2" t="inlineStr">
         <is>
@@ -5937,10 +6085,14 @@
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O77" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P77" s="2" t="n"/>
       <c r="Q77" s="2" t="n"/>
     </row>
@@ -6010,10 +6162,14 @@
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O78" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P78" s="2" t="n"/>
       <c r="Q78" s="2" t="n"/>
     </row>
@@ -6083,10 +6239,14 @@
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O79" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P79" s="2" t="n"/>
       <c r="Q79" s="2" t="inlineStr">
         <is>
@@ -6160,10 +6320,14 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O80" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P80" s="2" t="n"/>
       <c r="Q80" s="2" t="inlineStr">
         <is>
@@ -6237,10 +6401,14 @@
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O81" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P81" s="2" t="n"/>
       <c r="Q81" s="2" t="inlineStr">
         <is>
@@ -6302,10 +6470,14 @@
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O82" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P82" s="2" t="n"/>
       <c r="Q82" s="2" t="n"/>
     </row>
@@ -6375,10 +6547,14 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O83" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P83" s="2" t="n"/>
       <c r="Q83" s="2" t="inlineStr">
         <is>
@@ -6440,10 +6616,14 @@
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O84" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P84" s="2" t="n"/>
       <c r="Q84" s="2" t="n"/>
     </row>
@@ -6501,10 +6681,14 @@
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O85" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P85" s="2" t="n"/>
       <c r="Q85" s="2" t="n"/>
     </row>
@@ -6562,10 +6746,14 @@
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O86" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P86" s="2" t="n"/>
       <c r="Q86" s="2" t="n"/>
     </row>
@@ -6635,10 +6823,14 @@
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O87" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P87" s="2" t="n"/>
       <c r="Q87" s="2" t="n"/>
     </row>
@@ -6696,10 +6888,14 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O88" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P88" s="2" t="n"/>
       <c r="Q88" s="2" t="n"/>
     </row>
@@ -6769,10 +6965,14 @@
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O89" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P89" s="2" t="n"/>
       <c r="Q89" s="2" t="inlineStr">
         <is>
@@ -6846,10 +7046,14 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O90" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P90" s="2" t="n"/>
       <c r="Q90" s="2" t="inlineStr">
         <is>
@@ -6911,10 +7115,14 @@
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O91" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P91" s="2" t="n"/>
       <c r="Q91" s="2" t="n"/>
     </row>
@@ -6972,10 +7180,14 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O92" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P92" s="2" t="n"/>
       <c r="Q92" s="2" t="n"/>
     </row>
@@ -7045,10 +7257,14 @@
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O93" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P93" s="2" t="n"/>
       <c r="Q93" s="2" t="n"/>
     </row>
@@ -7118,10 +7334,14 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O94" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P94" s="2" t="n"/>
       <c r="Q94" s="2" t="inlineStr">
         <is>
@@ -7195,10 +7415,14 @@
       </c>
       <c r="N95" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O95" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P95" s="2" t="n"/>
       <c r="Q95" s="2" t="inlineStr">
         <is>
@@ -7272,10 +7496,14 @@
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O96" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P96" s="2" t="n"/>
       <c r="Q96" s="2" t="n"/>
     </row>
@@ -7333,10 +7561,14 @@
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O97" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P97" s="2" t="n"/>
       <c r="Q97" s="2" t="n"/>
     </row>
@@ -7463,10 +7695,14 @@
       </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O99" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="P99" s="2" t="n"/>
       <c r="Q99" s="2" t="n"/>
     </row>
@@ -7536,10 +7772,14 @@
       </c>
       <c r="N100" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O100" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P100" s="2" t="n"/>
       <c r="Q100" s="2" t="inlineStr">
         <is>
@@ -7613,10 +7853,14 @@
       </c>
       <c r="N101" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O101" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P101" s="2" t="n"/>
       <c r="Q101" s="2" t="n"/>
     </row>
@@ -7686,10 +7930,14 @@
       </c>
       <c r="N102" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O102" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P102" s="2" t="n"/>
       <c r="Q102" s="2" t="n"/>
     </row>
@@ -7747,10 +7995,14 @@
       </c>
       <c r="N103" s="2" t="inlineStr">
         <is>
-          <t>Not yet contacted</t>
-        </is>
-      </c>
-      <c r="O103" s="2" t="n"/>
+          <t>Emailed</t>
+        </is>
+      </c>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="P103" s="2" t="n"/>
       <c r="Q103" s="2" t="n"/>
     </row>
@@ -8799,7 +9051,7 @@
 Thanks for being part of this from early on,
 Ronnie Bouchon
 SaveTheHives — savethehives.org
-hello@savethehives.org</t>
+ronniebouchon@gmail.com</t>
         </is>
       </c>
     </row>

</xml_diff>